<commit_message>
Rework instructions and demo trials, add timeout message and Check button
- New intro flow (pages 1-10) with per-layer sound buttons (2 hits on beats
  1 and 3) and highlighted layer; texts in DMT_dict (en/de/de_f)
- Demo trials now mirror main trials (no solution preview, timer, both
  play buttons); num_examples defaults to 4 and is validated
- trial_timeout now applies to demo and main trials
- Show "Time is up!" in feedback on timeout; fix dmtTimedOut never being
  sent to R (timed_out was always FALSE)
- Trial input pages use "Check"/"Auflösung" instead of "Next"
- Load Tone.js only once, reuse samples, translate stop-button labels

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/DMT_dict.xlsx
+++ b/data-raw/DMT_dict.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Now you're ready for the real thing. Good luck!</t>
+          <t>Now you're ready for the real test. Good luck!</t>
         </is>
       </c>
     </row>
@@ -1473,6 +1473,732 @@
       <c r="D51" t="inlineStr">
         <is>
           <t>Continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>INSTR_WELCOME_TITLE</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Willkommen beim Drum Machine Test!</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Willkommen beim Drum Machine Test!</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Welcome to the Drum Machine Test!</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>INSTR_WELCOME_1</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Dies ist ein musikalischer Lerntest.</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Dies ist ein musikalischer Lerntest.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>This is a musical learning test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>INSTR_WELCOME_2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Du lernst, ein digitales Instrument zu bedienen: eine Drum Machine.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Sie lernen, ein digitales Instrument zu bedienen: eine Drum Machine.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>You will learn how to use a digital instrument: a drum machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>INSTR_TASK_TITLE</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Deine Aufgabe:</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Ihre Aufgabe:</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Your task:</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>INSTR_TASK_1</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Du hörst einen Rhythmus, den du auf der Drum Machine nachbauen sollst.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Sie hören einen Rhythmus, den Sie auf der Drum Machine nachbauen sollen.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>You will hear a rhythm which you have to recreate on the drum machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>INSTR_TASK_FEEDBACK</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Du bekommst Feedback zu deiner Leistung, damit du lernst, die Drum Machine zu bedienen.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Sie erhalten Feedback zu Ihrer Leistung, damit Sie lernen, die Drum Machine zu bedienen.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>You will receive feedback on how you perform to help you learn how to use the drum machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>INSTR_NAVIGATE</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Du kannst dich durch den Test bewegen, indem du auf „Weiter“ klickst.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Sie können sich durch den Test bewegen, indem Sie auf „Weiter“ klicken.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>You can navigate through the test by clicking "Continue".</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>INSTR_LEARNING_1</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Dies ist ein Lerntest – mach dir also keine Sorgen, wenn du den Rhythmus am Anfang nicht perfekt nachbauen kannst.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Dies ist ein Lerntest – machen Sie sich also keine Sorgen, wenn Sie den Rhythmus am Anfang nicht perfekt nachbauen können.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>This is a learning test, so don't worry if you can't recreate the rhythm perfectly in the beginning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>INSTR_LEARNING_2</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Der Test erklärt dir, wie die Drum Machine funktioniert.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Der Test erklärt Ihnen, wie die Drum Machine funktioniert.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>The test will instruct you on how the drum machine works.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>INSTR_LEARNING_3</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Zuerst erklären wir dir, wie die Drum Machine funktioniert:</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Zuerst erklären wir Ihnen, wie die Drum Machine funktioniert:</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>First, let's explain how the drum machine works:</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>INSTR_LOOKS_LIKE</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>So sieht die Drum Machine aus:</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>So sieht die Drum Machine aus:</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>This is what the drum machine looks like:</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>INSTR_LAYERS_INTRO</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Die Drum Machine besteht aus drei Ebenen:</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Die Drum Machine besteht aus drei Ebenen:</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>The drum machine consists of three layers:</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>INSTR_LAYER_1_TITLE</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1. Ebene: Hi-Hat</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1. Ebene: Hi-Hat</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>1st layer: Hi-hat</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>INSTR_LAYER_2_TITLE</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2. Ebene: Snare</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2. Ebene: Snare</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>2nd layer: Snare</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>INSTR_LAYER_3_TITLE</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>3. Ebene: Bassdrum</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>3. Ebene: Bassdrum</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>3rd layer: Bass drum</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>INSTR_LAYER_SOUNDS_LIKE</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>So klingt sie:</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>So klingt sie:</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>It sounds like this:</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>INSTR_EXPLORE_1</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Du aktivierst einen Klang, indem du auf ein Feld drückst.</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Sie aktivieren einen Klang, indem Sie auf ein Feld drücken.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>You enable a sound by pressing on the square.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>INSTR_EXPLORE_2</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Probiere gerne aus, wie die Drum Machine funktioniert.</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Probieren Sie gerne aus, wie die Drum Machine funktioniert.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Feel free to explore how the drum machine works.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>INSTR_EXPLORE_3</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Mit „Dein Muster abspielen“ kannst du hören, was du erstellt hast.</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Mit „Ihr Muster abspielen“ können Sie hören, was Sie erstellt haben.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>With "Play your pattern" you can listen to what you created.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>INSTR_FEEDBACK_1</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Du bekommst Feedback, wenn du den Rhythmus nicht perfekt nachbauen kannst.</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Sie erhalten Feedback, wenn Sie den Rhythmus nicht perfekt nachbauen können.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>You will receive feedback if you can't reproduce the rhythm perfectly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>INSTR_FEEDBACK_2</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Je öfter du einen Fehler machst, desto detaillierter wird das Feedback.</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Je öfter Sie einen Fehler machen, desto detaillierter wird das Feedback.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>The more often you make a mistake, the more detailed the feedback gets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>INSTR_PRACTICE_1</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Vor der eigentlichen Aufgabe absolvierst du ein paar Übungsdurchgänge, um die Drum Machine kennenzulernen.</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Vor der eigentlichen Aufgabe absolvieren Sie ein paar Übungsdurchgänge, um die Drum Machine kennenzulernen.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Before the main task, you will complete a few practice trials to get to know the drum machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>INSTR_PRACTICE_TIMER</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Du hast {{trial_timeout}} Sekunden Zeit, um das Muster nachzubauen.</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Sie haben {{trial_timeout}} Sekunden Zeit, um das Muster nachzubauen.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>You have {{trial_timeout}} seconds to recreate the pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>INSTR_EXAMPLE1_1</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Jetzt hörst du den ersten Rhythmus.</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Jetzt hören Sie den ersten Rhythmus.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Now you will hear the first rhythm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>INSTR_EXAMPLE1_2</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Mit dem Button „Stimulus abspielen“ kannst du dir den Rhythmus anhören, den du nachbauen sollst.</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Mit dem Button „Stimulus abspielen“ können Sie sich den Rhythmus anhören, den Sie nachbauen sollen.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>You can press the button "Play stimulus" to listen to the rhythm you have to recreate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>INSTR_EXAMPLE1_3</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Mit dem Button „Dein Muster abspielen“ kannst du dir anhören, was du erstellt hast.</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Mit dem Button „Ihr Muster abspielen“ können Sie sich anhören, was Sie erstellt haben.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>By pressing the button "Play your pattern", you can listen to what you created.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>BUTTON_STOP_STIMULUS</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Stimulus stoppen</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Stimulus stoppen</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Stop stimulus</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>BUTTON_STOP_PATTERN</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Dein Muster stoppen</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Ihr Muster stoppen</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Stop your pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>INSTR_SOUND_BUTTON_1</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Hi-Hat-Klang abspielen</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Hi-Hat-Klang abspielen</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Play Hi-hat sound</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>INSTR_SOUND_BUTTON_2</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Snare-Klang abspielen</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Snare-Klang abspielen</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Play Snare sound</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>INSTR_SOUND_BUTTON_3</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Bassdrum-Klang abspielen</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Bassdrum-Klang abspielen</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Play Bass drum sound</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>BUTTON_CHECK</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Auflösung</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Auflösung</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>FEEDBACK_TIME_UP</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Die Zeit ist abgelaufen!</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Die Zeit ist abgelaufen!</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Time is up!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Two practice trials, shorter instruction sentences, fix layer numbering
- num_examples default 4 -> 2; practice order Easy_1 (kick on 1+3),
  then new Practice_2 (kick 1, snare 2+4, hi-hat 3), added to
  demo_drum_matrix via data-raw/practice_stimuli.R (main pools unchanged)
- Shorten 9 instruction sentences (en/de/de_f); page structure unchanged
- Fix layer pages always showing "1.": custom CSS list counter ignored
  <ol start>
- Local test app: German, default practice trials

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/DMT_dict.xlsx
+++ b/data-raw/DMT_dict.xlsx
@@ -1594,17 +1594,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Du bekommst Feedback zu deiner Leistung, damit du lernst, die Drum Machine zu bedienen.</t>
+          <t>Du bekommst Feedback, das dir beim Lernen hilft.</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Sie erhalten Feedback zu Ihrer Leistung, damit Sie lernen, die Drum Machine zu bedienen.</t>
+          <t>Sie erhalten Feedback, das Ihnen beim Lernen hilft.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>You will receive feedback on how you perform to help you learn how to use the drum machine.</t>
+          <t>You will receive feedback that helps you learn.</t>
         </is>
       </c>
     </row>
@@ -1616,17 +1616,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Du kannst dich durch den Test bewegen, indem du auf „Weiter“ klickst.</t>
+          <t>Mit „Weiter“ kommst du zur nächsten Seite.</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sie können sich durch den Test bewegen, indem Sie auf „Weiter“ klicken.</t>
+          <t>Mit „Weiter“ kommen Sie zur nächsten Seite.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>You can navigate through the test by clicking "Continue".</t>
+          <t>Click "Continue" to go to the next page.</t>
         </is>
       </c>
     </row>
@@ -1638,17 +1638,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Dies ist ein Lerntest – mach dir also keine Sorgen, wenn du den Rhythmus am Anfang nicht perfekt nachbauen kannst.</t>
+          <t>Das ist ein Lerntest. Keine Sorge, wenn es am Anfang noch nicht klappt.</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Dies ist ein Lerntest – machen Sie sich also keine Sorgen, wenn Sie den Rhythmus am Anfang nicht perfekt nachbauen können.</t>
+          <t>Das ist ein Lerntest. Keine Sorge, wenn es am Anfang noch nicht klappt.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>This is a learning test, so don't worry if you can't recreate the rhythm perfectly in the beginning.</t>
+          <t>This is a learning test. Don't worry if it doesn't work out at first.</t>
         </is>
       </c>
     </row>
@@ -1880,17 +1880,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Mit „Dein Muster abspielen“ kannst du hören, was du erstellt hast.</t>
+          <t>Mit „Dein Muster abspielen“ hörst du, was du gebaut hast.</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Mit „Ihr Muster abspielen“ können Sie hören, was Sie erstellt haben.</t>
+          <t>Mit „Ihr Muster abspielen“ hören Sie, was Sie gebaut haben.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>With "Play your pattern" you can listen to what you created.</t>
+          <t>With "Play your pattern" you hear what you built.</t>
         </is>
       </c>
     </row>
@@ -1902,17 +1902,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Du bekommst Feedback, wenn du den Rhythmus nicht perfekt nachbauen kannst.</t>
+          <t>Wenn dein Rhythmus noch nicht stimmt, bekommst du Feedback.</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Sie erhalten Feedback, wenn Sie den Rhythmus nicht perfekt nachbauen können.</t>
+          <t>Wenn Ihr Rhythmus noch nicht stimmt, erhalten Sie Feedback.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>You will receive feedback if you can't reproduce the rhythm perfectly.</t>
+          <t>If your rhythm isn't right yet, you will receive feedback.</t>
         </is>
       </c>
     </row>
@@ -1924,17 +1924,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Je öfter du einen Fehler machst, desto detaillierter wird das Feedback.</t>
+          <t>Mit jedem Versuch wird das Feedback genauer.</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Je öfter Sie einen Fehler machen, desto detaillierter wird das Feedback.</t>
+          <t>Mit jedem Versuch wird das Feedback genauer.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>The more often you make a mistake, the more detailed the feedback gets.</t>
+          <t>The feedback gets more detailed with every attempt.</t>
         </is>
       </c>
     </row>
@@ -1946,17 +1946,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Vor der eigentlichen Aufgabe absolvierst du ein paar Übungsdurchgänge, um die Drum Machine kennenzulernen.</t>
+          <t>Zuerst lernst du die Drum Machine kennen.</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Vor der eigentlichen Aufgabe absolvieren Sie ein paar Übungsdurchgänge, um die Drum Machine kennenzulernen.</t>
+          <t>Zuerst lernen Sie die Drum Machine kennen.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Before the main task, you will complete a few practice trials to get to know the drum machine.</t>
+          <t>First, you will get to know the drum machine.</t>
         </is>
       </c>
     </row>
@@ -2012,17 +2012,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Mit dem Button „Stimulus abspielen“ kannst du dir den Rhythmus anhören, den du nachbauen sollst.</t>
+          <t>Mit „Stimulus abspielen“ hörst du den Rhythmus, den du nachbauen sollst.</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Mit dem Button „Stimulus abspielen“ können Sie sich den Rhythmus anhören, den Sie nachbauen sollen.</t>
+          <t>Mit „Stimulus abspielen“ hören Sie den Rhythmus, den Sie nachbauen sollen.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>You can press the button "Play stimulus" to listen to the rhythm you have to recreate.</t>
+          <t>With "Play stimulus" you hear the rhythm you have to recreate.</t>
         </is>
       </c>
     </row>
@@ -2034,17 +2034,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Mit dem Button „Dein Muster abspielen“ kannst du dir anhören, was du erstellt hast.</t>
+          <t>Mit „Dein Muster abspielen“ hörst du, was du gebaut hast.</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Mit dem Button „Ihr Muster abspielen“ können Sie sich anhören, was Sie erstellt haben.</t>
+          <t>Mit „Ihr Muster abspielen“ hören Sie, was Sie gebaut haben.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>By pressing the button "Play your pattern", you can listen to what you created.</t>
+          <t>With "Play your pattern" you hear what you built.</t>
         </is>
       </c>
     </row>

</xml_diff>